<commit_message>
feat: auto-open room interactions and waive first room fee
</commit_message>
<xml_diff>
--- a/config/excel/CfgGuide.xlsx
+++ b/config/excel/CfgGuide.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgGuide" sheetId="1" r:id="Rc72638a6cf8e4473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgGuide" sheetId="1" r:id="R030fbb219f39463b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,29 +13,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
+  <x:fonts count="1">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="2">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF17365D"/>
-      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="1">
@@ -50,10 +39,8 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="3">
+  <x:cellXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -257,16 +244,16 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="2" t="str">
+      <x:c r="A1" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="B1" s="2" t="str">
+      <x:c r="B1" t="str">
         <x:v>SortOrder</x:v>
       </x:c>
-      <x:c r="C1" s="2" t="str">
+      <x:c r="C1" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="D1" s="2" t="str">
+      <x:c r="D1" t="str">
         <x:v>Body</x:v>
       </x:c>
     </x:row>
@@ -295,7 +282,7 @@
         <x:v>移动与战斗</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>拖动摇杆移动角色，敌人进入近战范围后自动攻击。留意生命值和地面预警，完成当前房间目标后向上方出口前进。</x:v>
+        <x:v>拖动摇杆移动角色，敌人进入近战范围后自动攻击。触碰NPC、未领取宝箱或已开放出口时自动打开对应窗口并暂停战斗，无需按键或点击主界面互动按钮。留意生命值和地面预警，完成当前房间目标后向上方出口前进。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -309,7 +296,7 @@
         <x:v>线性房间关卡</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>房间按顺序单向推进，最后为Boss房；怪物房清场后开放出口，最终Boss奖励领取完毕后通关并带回收益。当前六房排列是可调原型，包含怪物房、宝箱房和商人房。</x:v>
+        <x:v>房间按顺序单向推进，最后为Boss房；怪物房清场后开放出口，最终Boss奖励领取完毕后自动通关并带回收益。关闭NPC或出口窗口后，先离开触碰范围，再进入即可重新打开；站在原地不会反复弹窗，宝箱领取后不再触发。当前六房排列是可调原型，包含怪物房、宝箱房和商人房。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -379,7 +366,7 @@
         <x:v>入场体力与补给</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>首次开启关卡消耗{EntryCost}点体力，每次进入房间消耗{RoomEntryCost}点；继续宝箱房不额外扣费，重新进入未完成怪物或Boss房仍消耗{RoomEntryCost}点。体力上限{StaminaCap}点，每{RecoverySeconds}秒恢复1点，每天{DailyResetHour}点重置到上限。每天{SupplyHourFirst}点、{SupplyHourSecond}点、{SupplyHourThird}点可手动领取{SupplyAmount}点补给。</x:v>
+        <x:v>首次开启关卡只消耗{EntryCost}点体力，第一房不另收费；后续每进入一个新房间消耗{RoomEntryCost}点。继续宝箱房不扣费，继续未完成怪物或Boss房消耗{RoomEntryCost}点；NPC房续关直接进入下一房并消耗{RoomEntryCost}点。最终Boss已全部领奖、仅待补办通关时恢复免费。体力上限{StaminaCap}点，每{RecoverySeconds}秒恢复1点，每天{DailyResetHour}点重置到上限。每天{SupplyHourFirst}点、{SupplyHourSecond}点、{SupplyHourThird}点可手动领取{SupplyAmount}点补给。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: add boss reward chests and explicit final exit
</commit_message>
<xml_diff>
--- a/config/excel/CfgGuide.xlsx
+++ b/config/excel/CfgGuide.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgGuide" sheetId="1" r:id="R030fbb219f39463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgGuide" sheetId="1" r:id="Rd4616a990aaa4dc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -296,7 +296,7 @@
         <x:v>线性房间关卡</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>房间按顺序单向推进，最后为Boss房；怪物房清场后开放出口，最终Boss奖励领取完毕后自动通关并带回收益。关闭NPC或出口窗口后，先离开触碰范围，再进入即可重新打开；站在原地不会反复弹窗，宝箱领取后不再触发。当前六房排列是可调原型，包含怪物房、宝箱房和商人房。</x:v>
+        <x:v>房间按顺序单向推进，最后为Boss房；怪物房清场后开放出口。最终Boss击败后出现奖励宝箱，触碰开启后按原有轮次选择战利品，全部领取后开放上方出口；触碰最终出口打开结算对话框，确认后通关并带回收益。关闭NPC或出口窗口后，先离开触碰范围，再进入即可重新打开；站在原地不会反复弹窗，已领取完的宝箱不再触发。当前六房排列是可调原型，包含怪物房、宝箱房和商人房。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -352,7 +352,7 @@
         <x:v>暂离与继续</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>暂离主城保留关卡背包、角色收益和消耗。未完成的怪物或Boss战再次进入时重开，已确认的敌人收益不重复发放。未领取完的宝箱房保留；离开NPC房后继续下一房。已击败Boss但尚未领奖时继续处理原奖励。</x:v>
+        <x:v>暂离主城保留关卡背包、角色收益和消耗。未完成的怪物或Boss战再次进入时重开，已确认的敌人收益不重复发放。未领取完的宝箱房保留；离开NPC房后继续下一房。最终Boss已击败但宝箱未开或奖励未领完时，继续回到本房领取，敌人不重生，冻结候选与已领取事实保留；全部领奖后仍需走到出口确认结算。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -366,7 +366,7 @@
         <x:v>入场体力与补给</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>首次开启关卡只消耗{EntryCost}点体力，第一房不另收费；后续每进入一个新房间消耗{RoomEntryCost}点。继续宝箱房不扣费，继续未完成怪物或Boss房消耗{RoomEntryCost}点；NPC房续关直接进入下一房并消耗{RoomEntryCost}点。最终Boss已全部领奖、仅待补办通关时恢复免费。体力上限{StaminaCap}点，每{RecoverySeconds}秒恢复1点，每天{DailyResetHour}点重置到上限。每天{SupplyHourFirst}点、{SupplyHourSecond}点、{SupplyHourThird}点可手动领取{SupplyAmount}点补给。</x:v>
+        <x:v>首次开启关卡只消耗{EntryCost}点体力，第一房不另收费；后续每进入一个新房间消耗{RoomEntryCost}点。继续宝箱房不扣费，继续未完成怪物或Boss战消耗{RoomEntryCost}点；NPC房续关直接进入下一房并消耗{RoomEntryCost}点。最终Boss已击败后的宝箱领取及出口结算阶段继续免费，死亡待选仍须按原选择处理。体力上限{StaminaCap}点，每{RecoverySeconds}秒恢复1点，每天{DailyResetHour}点重置到上限。每天{SupplyHourFirst}点、{SupplyHourSecond}点、{SupplyHourThird}点可手动领取{SupplyAmount}点补给。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: claim all boss chest rewards at once
</commit_message>
<xml_diff>
--- a/config/excel/CfgGuide.xlsx
+++ b/config/excel/CfgGuide.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgGuide" sheetId="1" r:id="Rd4616a990aaa4dc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CfgGuide" sheetId="1" r:id="R4272c080b5194b7d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -296,7 +296,7 @@
         <x:v>线性房间关卡</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>房间按顺序单向推进，最后为Boss房；怪物房清场后开放出口。最终Boss击败后出现奖励宝箱，触碰开启后按原有轮次选择战利品，全部领取后开放上方出口；触碰最终出口打开结算对话框，确认后通关并带回收益。关闭NPC或出口窗口后，先离开触碰范围，再进入即可重新打开；站在原地不会反复弹窗，已领取完的宝箱不再触发。当前六房排列是可调原型，包含怪物房、宝箱房和商人房。</x:v>
+        <x:v>房间按顺序单向推进，最后为Boss房；怪物房清场后开放出口。最终Boss击败后出现奖励宝箱，触碰开启后展示本箱已经冻结的全部物品，只需点击一次领取按钮即可全部获得，不逐件选择、不分轮。领取完成后开放上方出口；触碰最终出口打开结算对话框，确认后通关并带回收益。关闭NPC、未领宝箱或出口窗口后，先离开触碰范围再进入可重新打开，站在原地不反复弹窗，已领取宝箱不再触发。当前六房排列是可调原型。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -352,7 +352,7 @@
         <x:v>暂离与继续</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>暂离主城保留关卡背包、角色收益和消耗。未完成的怪物或Boss战再次进入时重开，已确认的敌人收益不重复发放。未领取完的宝箱房保留；离开NPC房后继续下一房。最终Boss已击败但宝箱未开或奖励未领完时，继续回到本房领取，敌人不重生，冻结候选与已领取事实保留；全部领奖后仍需走到出口确认结算。</x:v>
+        <x:v>暂离主城保留关卡背包、角色收益和消耗。未完成的怪物或Boss战再次进入时重开，已确认的敌人收益不重复发放。未领取完的宝箱房保留；离开NPC房后继续下一房。最终Boss已击败但宝箱未开或尚未领取时，继续回到本房领取，敌人不重生，整箱冻结物品保持不变；一键领取全部后仍需走到出口确认结算。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>